<commit_message>
Put the sample customer list back to the generated ten
The committed customers_dummy.xlsx had been trimmed to two rows with real numbers for a live test,
which is what backend/local/ is for: fixtures are sample data every checkout shares, and a real
WhatsApp number in git is permanent in a way a wrong one in a test is not. The file is the generated
ten again, so test_the_committed_sample_data_is_the_generated_one passes and the dummy data matches
the orders it is meant to line up with.

The live copy is untouched, in backend/local/, which is git-ignored; CUSTOMERS_FILE_PATH points at
whichever of the two the bot should read.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/fixtures/customers_dummy.xlsx
+++ b/backend/fixtures/customers_dummy.xlsx
@@ -1,64 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Customers" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
-  <si>
-    <t>Customer Code</t>
-  </si>
-  <si>
-    <t>Customer Name</t>
-  </si>
-  <si>
-    <t>Contact</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>C001</t>
-  </si>
-  <si>
-    <t>Shree Packaging Pvt Ltd</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>C002</t>
-  </si>
-  <si>
-    <t>Mehta Foods</t>
-  </si>
-  <si>
-    <t>+91 9924517622</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -77,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -170,7 +199,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -205,7 +233,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -240,16 +267,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -371,113 +402,318 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="13.571428571428571" customWidth="1"/>
-    <col min="2" max="2" width="17.428571428571427" customWidth="1"/>
-    <col min="3" max="3" width="19.571428571428573" customWidth="1"/>
-    <col min="4" max="24" width="13.571428571428571" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>9199988877765</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Customer Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Customer Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Shree Packaging Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>9167861236</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>shree@example.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mehta Foods</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+91 98765-43210</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mehta@example.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gujarat Polymers</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>09898012345</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>gp@example.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Patel Agro Industries</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>91 9925001122</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>patel@example.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sunrise Pharma</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>9033445566</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>sun@example.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Royal Textiles</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>+919712345678</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>royal@example.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Anand Dairy Products</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>9081726354</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>anand@example.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Om Snacks</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>9427000111</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>om@example.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bad Number Co</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>98765</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>bad@example.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Duplicate Co</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>9167861236</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>dup@example.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>